<commit_message>
12.1.1 se actualizaron las matrices para incorporar nuevos parametos
</commit_message>
<xml_diff>
--- a/static/excel_files/pruebas_corr_datos_stv_evolutivo_admin.xlsx
+++ b/static/excel_files/pruebas_corr_datos_stv_evolutivo_admin.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="23">
   <si>
     <t xml:space="preserve">Alcance Evaluación</t>
   </si>
@@ -31,13 +31,25 @@
     <t xml:space="preserve">Fase</t>
   </si>
   <si>
-    <t xml:space="preserve">Caso de prueba</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Críticidad</t>
+    <t xml:space="preserve">caso de prueba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Criticidad</t>
   </si>
   <si>
     <t xml:space="preserve">nota sobre la prueba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">etiqueta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tipo de usuario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pasos</t>
   </si>
   <si>
     <t xml:space="preserve">A</t>
@@ -89,7 +101,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -121,6 +133,20 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Comfortaa"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Comfortaa"/>
@@ -137,8 +163,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF26A69A"/>
-        <bgColor rgb="FF33CCCC"/>
+        <fgColor rgb="FF069A2E"/>
+        <bgColor rgb="FF339966"/>
       </patternFill>
     </fill>
     <fill>
@@ -188,7 +214,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -201,27 +227,43 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -238,7 +280,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FF26A69A"/>
+          <fgColor rgb="FF069A2E"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -343,7 +385,7 @@
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FF00FFFF"/>
       <rgbColor rgb="FF660000"/>
-      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF069A2E"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FF7F6000"/>
       <rgbColor rgb="FF800080"/>
@@ -383,7 +425,7 @@
       <rgbColor rgb="FF666699"/>
       <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF003366"/>
-      <rgbColor rgb="FF26A69A"/>
+      <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF003300"/>
       <rgbColor rgb="FF333300"/>
       <rgbColor rgb="FF783F04"/>
@@ -577,7 +619,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H1048576"/>
+  <dimension ref="A1:I1048576"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15"/>
@@ -599,335 +641,345 @@
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2"/>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
       <c r="E1" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
+      <c r="B2" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="6"/>
     </row>
     <row r="3" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="6" t="s">
+      <c r="A3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="5" t="s">
+      <c r="C3" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="8"/>
+    </row>
+    <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
-      <c r="H3" s="6"/>
-    </row>
-    <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="3" t="s">
+      <c r="B4" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="10"/>
+      <c r="G4" s="10"/>
+      <c r="H4" s="10"/>
+    </row>
+    <row r="5" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-    </row>
-    <row r="5" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" s="6" t="s">
+      <c r="B5" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="8"/>
+      <c r="G5" s="8"/>
+      <c r="H5" s="8"/>
+    </row>
+    <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
-      <c r="H5" s="6"/>
-    </row>
-    <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" s="4" t="s">
+      <c r="B6" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" s="3" t="s">
+      <c r="F6" s="10"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
+    </row>
+    <row r="7" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
-    </row>
-    <row r="7" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E7" s="5" t="s">
+      <c r="B7" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
+    </row>
+    <row r="8" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
-    </row>
-    <row r="8" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E8" s="3" t="s">
+      <c r="B8" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
+    </row>
+    <row r="9" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4"/>
-    </row>
-    <row r="9" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E9" s="5" t="s">
+      <c r="B9" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
+    </row>
+    <row r="10" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
-      <c r="H9" s="6"/>
-    </row>
-    <row r="10" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E10" s="3" t="s">
+      <c r="B10" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10" s="10"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="10"/>
+    </row>
+    <row r="11" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
-    </row>
-    <row r="11" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
+      <c r="B11" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
+      <c r="A12" s="9"/>
+      <c r="B12" s="9"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="10"/>
+      <c r="H12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5"/>
-      <c r="B13" s="5"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
-      <c r="H13" s="6"/>
+      <c r="A13" s="7"/>
+      <c r="B13" s="7"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3"/>
-      <c r="B14" s="3"/>
-      <c r="C14" s="4"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
+      <c r="A14" s="9"/>
+      <c r="B14" s="9"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="10"/>
+      <c r="H14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5"/>
-      <c r="B15" s="5"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="6"/>
+      <c r="A15" s="7"/>
+      <c r="B15" s="7"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8"/>
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5"/>
-      <c r="B16" s="5"/>
-      <c r="C16" s="6"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="6"/>
-      <c r="G16" s="6"/>
-      <c r="H16" s="6"/>
+      <c r="A16" s="7"/>
+      <c r="B16" s="7"/>
+      <c r="C16" s="8"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="8"/>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3"/>
-      <c r="B17" s="3"/>
-      <c r="C17" s="4"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="4"/>
-      <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
+      <c r="A17" s="9"/>
+      <c r="B17" s="9"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="10"/>
+      <c r="H17" s="10"/>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3"/>
-      <c r="B18" s="3"/>
-      <c r="C18" s="4"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="4"/>
-      <c r="G18" s="4"/>
-      <c r="H18" s="4"/>
+      <c r="A18" s="9"/>
+      <c r="B18" s="9"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="10"/>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5"/>
-      <c r="B19" s="5"/>
-      <c r="C19" s="6"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="6"/>
-      <c r="G19" s="6"/>
-      <c r="H19" s="6"/>
+      <c r="A19" s="7"/>
+      <c r="B19" s="7"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="8"/>
+      <c r="H19" s="8"/>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="5"/>
-      <c r="B20" s="5"/>
-      <c r="C20" s="6"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="6"/>
-      <c r="G20" s="6"/>
-      <c r="H20" s="6"/>
+      <c r="A20" s="7"/>
+      <c r="B20" s="7"/>
+      <c r="C20" s="8"/>
+      <c r="D20" s="7"/>
+      <c r="E20" s="7"/>
+      <c r="F20" s="8"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="8"/>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5"/>
-      <c r="B21" s="5"/>
-      <c r="C21" s="6"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="6"/>
-      <c r="G21" s="6"/>
-      <c r="H21" s="6"/>
+      <c r="A21" s="7"/>
+      <c r="B21" s="7"/>
+      <c r="C21" s="8"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
+      <c r="F21" s="8"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="8"/>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="5"/>
-      <c r="B22" s="5"/>
-      <c r="C22" s="6"/>
-      <c r="D22" s="5"/>
-      <c r="E22" s="5"/>
-      <c r="F22" s="6"/>
-      <c r="G22" s="6"/>
-      <c r="H22" s="6"/>
+      <c r="A22" s="7"/>
+      <c r="B22" s="7"/>
+      <c r="C22" s="8"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7"/>
+      <c r="F22" s="8"/>
+      <c r="G22" s="8"/>
+      <c r="H22" s="8"/>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="5"/>
-      <c r="B23" s="5"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="5"/>
-      <c r="E23" s="5"/>
-      <c r="F23" s="6"/>
-      <c r="G23" s="6"/>
-      <c r="H23" s="6"/>
+      <c r="A23" s="7"/>
+      <c r="B23" s="7"/>
+      <c r="C23" s="8"/>
+      <c r="D23" s="7"/>
+      <c r="E23" s="7"/>
+      <c r="F23" s="8"/>
+      <c r="G23" s="8"/>
+      <c r="H23" s="8"/>
     </row>
     <row r="1048300" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048301" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -1225,6 +1277,40 @@
       <formula>NOT(ISERROR(SEARCH("Por ejecutar",D2)))</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="D2:E2">
+    <cfRule type="containsText" priority="7" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="Funciona" dxfId="6">
+      <formula>NOT(ISERROR(SEARCH("Funciona",D2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="8" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="Falla" dxfId="7">
+      <formula>NOT(ISERROR(SEARCH("Falla",D2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="9" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="N/A" dxfId="8">
+      <formula>NOT(ISERROR(SEARCH("N/A",D2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="10" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="Pendiente" dxfId="9">
+      <formula>NOT(ISERROR(SEARCH("Pendiente",D2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="11" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="Por ejecutar" dxfId="10">
+      <formula>NOT(ISERROR(SEARCH("Por ejecutar",D2)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D2:E2">
+    <cfRule type="containsText" priority="12" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="Funciona" dxfId="6">
+      <formula>NOT(ISERROR(SEARCH("Funciona",D2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="13" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="Falla" dxfId="7">
+      <formula>NOT(ISERROR(SEARCH("Falla",D2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="14" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="N/A" dxfId="8">
+      <formula>NOT(ISERROR(SEARCH("N/A",D2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="15" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="Pendiente" dxfId="9">
+      <formula>NOT(ISERROR(SEARCH("Pendiente",D2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="16" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="Por ejecutar" dxfId="10">
+      <formula>NOT(ISERROR(SEARCH("Por ejecutar",D2)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="4">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="A2:A23" type="list">
       <formula1>"A,B,C"</formula1>

</xml_diff>